<commit_message>
Fix main loader hang from malformed talent replacement data
Three talents (1004, 1011, 1028) had unquoted `[3,XXXX]` cells in the
content-pack CSV; the comma inside the brackets split into a second
column, so the runtime saw `replacement` as the string `"[3"`. The
for-of in Talent.initial then tried to write to a string index and
threw — and because game.start() in index.js is fire-and-forget, the
rejection was swallowed and switchView(MAIN) never ran, leaving the
loading screen up forever.

- Quote the bracketed values in talents.csv and rebuild the xlsx/JSON.
- Make Talent.initial defensive: skip and warn on non-object
  replacement instead of crashing the whole init.
- Wrap core.initial in App.start with try/catch so future init errors
  surface in console and the main view still loads.
- Drop the hardcoded codex-runtimes Python path in
  build-content-pack-data.mjs; fall back to \$PYTHON or python3.
</commit_message>
<xml_diff>
--- a/data/en-us/talents.xlsx
+++ b/data/en-us/talents.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:R74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,7 +519,6 @@
           <t>replacement</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -592,7 +591,6 @@
           <t>替换规则</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -661,7 +659,6 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -722,7 +719,6 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -783,7 +779,6 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -845,12 +840,7 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>[3</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>1032]</t>
+          <t>[3,1032]</t>
         </is>
       </c>
     </row>
@@ -913,7 +903,6 @@
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -974,7 +963,6 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1035,7 +1023,6 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1096,7 +1083,6 @@
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1157,7 +1143,6 @@
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1218,7 +1203,6 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1280,12 +1264,7 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>[3</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>1065]</t>
+          <t>[3,1065]</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1331,6 @@
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1417,7 +1395,6 @@
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1478,7 +1455,6 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1539,7 +1515,6 @@
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1600,7 +1575,6 @@
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1661,7 +1635,6 @@
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1722,7 +1695,6 @@
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1783,7 +1755,6 @@
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1844,7 +1815,6 @@
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1905,7 +1875,6 @@
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1966,7 +1935,6 @@
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2027,7 +1995,6 @@
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2088,7 +2055,6 @@
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2149,7 +2115,6 @@
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2210,7 +2175,6 @@
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2271,7 +2235,6 @@
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2333,12 +2296,7 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>[3</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>1061]</t>
+          <t>[3,1061]</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2359,6 @@
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2462,7 +2419,6 @@
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2523,7 +2479,6 @@
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2588,7 +2543,6 @@
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2653,7 +2607,6 @@
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2718,7 +2671,6 @@
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2779,7 +2731,6 @@
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2840,7 +2791,6 @@
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2901,7 +2851,6 @@
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2962,7 +2911,6 @@
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3023,7 +2971,6 @@
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3084,7 +3031,6 @@
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3145,7 +3091,6 @@
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3210,7 +3155,6 @@
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3271,7 +3215,6 @@
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3332,7 +3275,6 @@
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3393,7 +3335,6 @@
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3454,7 +3395,6 @@
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3515,7 +3455,6 @@
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3576,7 +3515,6 @@
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3637,7 +3575,6 @@
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3698,7 +3635,6 @@
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3759,7 +3695,6 @@
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3824,7 +3759,6 @@
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3889,7 +3823,6 @@
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3950,7 +3883,6 @@
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4011,7 +3943,6 @@
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4072,7 +4003,6 @@
       <c r="P58" t="inlineStr"/>
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4133,7 +4063,6 @@
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4194,7 +4123,6 @@
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4255,7 +4183,6 @@
       <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4320,7 +4247,6 @@
       <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4381,7 +4307,6 @@
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4442,7 +4367,6 @@
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4503,7 +4427,6 @@
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4564,7 +4487,6 @@
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4629,7 +4551,6 @@
       <c r="P67" t="inlineStr"/>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4690,7 +4611,6 @@
       <c r="P68" t="inlineStr"/>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4755,7 +4675,6 @@
       <c r="P69" t="inlineStr"/>
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4816,7 +4735,6 @@
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4877,7 +4795,6 @@
       <c r="P71" t="inlineStr"/>
       <c r="Q71" t="inlineStr"/>
       <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4938,7 +4855,6 @@
       <c r="P72" t="inlineStr"/>
       <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4999,7 +4915,6 @@
       <c r="P73" t="inlineStr"/>
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5060,7 +4975,6 @@
       <c r="P74" t="inlineStr"/>
       <c r="Q74" t="inlineStr"/>
       <c r="R74" t="inlineStr"/>
-      <c r="S74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>